<commit_message>
a whole buncha stuff
</commit_message>
<xml_diff>
--- a/islamiceval/outputs/correction/corrections_complete_lenient_expansion.xlsx
+++ b/islamiceval/outputs/correction/corrections_complete_lenient_expansion.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/33c3ada92ee8b9a1/Desktop/dissertation/islamiceval/outputs/correction/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_B51800B1EAD1A3CC5088580AE4CDD70CAB4B0DD4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="corrections"/>
+    <sheet name="corrections" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -1438,8 +1444,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1450,7 +1455,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFffffff"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1487,17 +1492,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFe2efda"/>
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFfce4d6"/>
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFd9e1f2"/>
+        <fgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -1511,16 +1516,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </left>
       <right style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </right>
       <top style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFc6c6c6"/>
+        <color rgb="FFC6C6C6"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1535,86 +1540,66 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+  <cellXfs count="17">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1625,10 +1610,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -1666,71 +1651,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1758,7 +1743,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1781,11 +1766,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1794,13 +1779,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1810,7 +1795,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1819,7 +1804,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1828,7 +1813,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1836,10 +1821,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1904,28 +1889,27 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:L128"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" style="19" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="19" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="20" width="52.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="20" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="20" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="21" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="22" width="11.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="22" width="50.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="22" width="50.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="22" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="23" width="9.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="22" width="70.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="9" style="10" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" style="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52" style="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" style="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="11" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="50" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9" style="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="70" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="1" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1963,7 +1947,7 @@
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="72" customFormat="1" s="1">
+    <row r="2" spans="1:12" s="1" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
@@ -1995,7 +1979,7 @@
         <v>19</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="45.75" customFormat="1" s="1">
+    <row r="3" spans="1:12" s="1" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>20</v>
       </c>
@@ -2033,7 +2017,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="124.5" customFormat="1" s="1">
+    <row r="4" spans="1:12" s="1" customFormat="1" ht="124.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
         <v>25</v>
       </c>
@@ -2071,7 +2055,7 @@
         <v>30</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="98.25" customFormat="1" s="1">
+    <row r="5" spans="1:12" s="1" customFormat="1" ht="98.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>31</v>
       </c>
@@ -2109,7 +2093,7 @@
         <v>35</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row r="6" spans="1:12" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>36</v>
       </c>
@@ -2141,7 +2125,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="190.5" customFormat="1" s="1">
+    <row r="7" spans="1:12" s="1" customFormat="1" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
         <v>40</v>
       </c>
@@ -2179,7 +2163,7 @@
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="84.75" customFormat="1" s="1">
+    <row r="8" spans="1:12" s="1" customFormat="1" ht="84.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>45</v>
       </c>
@@ -2217,7 +2201,7 @@
         <v>49</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row r="9" spans="1:12" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
         <v>50</v>
       </c>
@@ -2249,7 +2233,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="72" customFormat="1" s="1">
+    <row r="10" spans="1:12" s="1" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
         <v>53</v>
       </c>
@@ -2283,7 +2267,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="72" customFormat="1" s="1">
+    <row r="11" spans="1:12" s="1" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>57</v>
       </c>
@@ -2321,7 +2305,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="111.75" customFormat="1" s="1">
+    <row r="12" spans="1:12" s="1" customFormat="1" ht="111.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>59</v>
       </c>
@@ -2359,7 +2343,7 @@
         <v>63</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="13" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>64</v>
       </c>
@@ -2391,7 +2375,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row r="14" spans="1:12" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
         <v>66</v>
       </c>
@@ -2429,7 +2413,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="32.25" customFormat="1" s="1">
+    <row r="15" spans="1:12" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
         <v>69</v>
       </c>
@@ -2461,7 +2445,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="150.75" customFormat="1" s="1">
+    <row r="16" spans="1:12" s="1" customFormat="1" ht="150.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>71</v>
       </c>
@@ -2495,7 +2479,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="17" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
         <v>71</v>
       </c>
@@ -2527,7 +2511,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="45.75" customFormat="1" s="1">
+    <row r="18" spans="1:12" s="1" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>64</v>
       </c>
@@ -2565,7 +2549,7 @@
         <v>78</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="204" customFormat="1" s="1">
+    <row r="19" spans="1:12" s="1" customFormat="1" ht="204" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
         <v>79</v>
       </c>
@@ -2597,7 +2581,7 @@
         <v>81</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="20" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
         <v>36</v>
       </c>
@@ -2629,7 +2613,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="45.75" customFormat="1" s="1">
+    <row r="21" spans="1:12" s="1" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>84</v>
       </c>
@@ -2661,7 +2645,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="22" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
         <v>84</v>
       </c>
@@ -2695,7 +2679,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="23" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>40</v>
       </c>
@@ -2727,7 +2711,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="24" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
         <v>89</v>
       </c>
@@ -2759,7 +2743,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="25" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
         <v>92</v>
       </c>
@@ -2791,7 +2775,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="26" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>94</v>
       </c>
@@ -2825,7 +2809,7 @@
         <v>97</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="27" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
         <v>98</v>
       </c>
@@ -2857,7 +2841,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="28" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>100</v>
       </c>
@@ -2889,7 +2873,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="29" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
         <v>102</v>
       </c>
@@ -2921,7 +2905,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="30" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
         <v>105</v>
       </c>
@@ -2955,7 +2939,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="31" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>84</v>
       </c>
@@ -2993,7 +2977,7 @@
         <v>110</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="32" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
         <v>31</v>
       </c>
@@ -3025,7 +3009,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="33" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>112</v>
       </c>
@@ -3057,7 +3041,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="34" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
         <v>114</v>
       </c>
@@ -3089,7 +3073,7 @@
         <v>118</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="35" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
         <v>119</v>
       </c>
@@ -3127,7 +3111,7 @@
         <v>123</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="36" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>50</v>
       </c>
@@ -3159,7 +3143,7 @@
         <v>126</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="37" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
         <v>57</v>
       </c>
@@ -3191,7 +3175,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="38" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>40</v>
       </c>
@@ -3223,7 +3207,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="39" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
         <v>129</v>
       </c>
@@ -3255,7 +3239,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="40" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
         <v>114</v>
       </c>
@@ -3289,7 +3273,7 @@
         <v>133</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="41" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>134</v>
       </c>
@@ -3323,7 +3307,7 @@
         <v>138</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="42" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
         <v>102</v>
       </c>
@@ -3357,7 +3341,7 @@
         <v>141</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="43" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
         <v>142</v>
       </c>
@@ -3389,7 +3373,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="44" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
         <v>144</v>
       </c>
@@ -3421,7 +3405,7 @@
         <v>146</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="45" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
         <v>147</v>
       </c>
@@ -3459,7 +3443,7 @@
         <v>151</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="46" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
         <v>142</v>
       </c>
@@ -3491,7 +3475,7 @@
         <v>153</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="47" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
         <v>154</v>
       </c>
@@ -3529,7 +3513,7 @@
         <v>157</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="48" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
         <v>158</v>
       </c>
@@ -3561,7 +3545,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="49" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
         <v>25</v>
       </c>
@@ -3593,7 +3577,7 @@
         <v>162</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="50" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
         <v>163</v>
       </c>
@@ -3625,7 +3609,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="51" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
         <v>57</v>
       </c>
@@ -3657,7 +3641,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="52" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
         <v>158</v>
       </c>
@@ -3689,7 +3673,7 @@
         <v>167</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="53" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
         <v>163</v>
       </c>
@@ -3721,7 +3705,7 @@
         <v>169</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="54" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
         <v>31</v>
       </c>
@@ -3753,7 +3737,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="55" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
         <v>25</v>
       </c>
@@ -3785,7 +3769,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="56" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
         <v>129</v>
       </c>
@@ -3817,7 +3801,7 @@
         <v>173</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="57" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
         <v>119</v>
       </c>
@@ -3849,7 +3833,7 @@
         <v>175</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="58" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
         <v>59</v>
       </c>
@@ -3881,7 +3865,7 @@
         <v>177</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="59" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
         <v>178</v>
       </c>
@@ -3913,7 +3897,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="60" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
         <v>180</v>
       </c>
@@ -3945,7 +3929,7 @@
         <v>182</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="61" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
         <v>183</v>
       </c>
@@ -3977,7 +3961,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="62" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
         <v>40</v>
       </c>
@@ -4011,7 +3995,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="63" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
         <v>114</v>
       </c>
@@ -4043,7 +4027,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="64" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
         <v>89</v>
       </c>
@@ -4075,7 +4059,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="65" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
         <v>189</v>
       </c>
@@ -4107,7 +4091,7 @@
         <v>191</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="66" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
         <v>144</v>
       </c>
@@ -4145,7 +4129,7 @@
         <v>194</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="67" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
         <v>94</v>
       </c>
@@ -4183,7 +4167,7 @@
         <v>198</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="68" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
         <v>50</v>
       </c>
@@ -4221,7 +4205,7 @@
         <v>202</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="69" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
         <v>203</v>
       </c>
@@ -4259,7 +4243,7 @@
         <v>206</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="70" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
         <v>59</v>
       </c>
@@ -4297,7 +4281,7 @@
         <v>210</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="71" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
         <v>211</v>
       </c>
@@ -4335,7 +4319,7 @@
         <v>215</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="72" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
         <v>216</v>
       </c>
@@ -4373,7 +4357,7 @@
         <v>219</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="73" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
         <v>220</v>
       </c>
@@ -4407,7 +4391,7 @@
         <v>223</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="74" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
         <v>189</v>
       </c>
@@ -4445,7 +4429,7 @@
         <v>226</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="75" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
         <v>69</v>
       </c>
@@ -4483,7 +4467,7 @@
         <v>194</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="76" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
         <v>45</v>
       </c>
@@ -4521,7 +4505,7 @@
         <v>230</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="77" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
         <v>94</v>
       </c>
@@ -4559,7 +4543,7 @@
         <v>233</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="78" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
         <v>134</v>
       </c>
@@ -4597,7 +4581,7 @@
         <v>236</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="79" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
         <v>237</v>
       </c>
@@ -4635,7 +4619,7 @@
         <v>240</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="80" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
         <v>241</v>
       </c>
@@ -4673,7 +4657,7 @@
         <v>244</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="81" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
         <v>20</v>
       </c>
@@ -4711,7 +4695,7 @@
         <v>247</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="82" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
         <v>241</v>
       </c>
@@ -4749,7 +4733,7 @@
         <v>250</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="83" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
         <v>180</v>
       </c>
@@ -4787,7 +4771,7 @@
         <v>253</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="84" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
         <v>158</v>
       </c>
@@ -4821,7 +4805,7 @@
         <v>256</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="85" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
         <v>180</v>
       </c>
@@ -4859,7 +4843,7 @@
         <v>260</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="86" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
         <v>261</v>
       </c>
@@ -4897,7 +4881,7 @@
         <v>265</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="87" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
         <v>189</v>
       </c>
@@ -4935,7 +4919,7 @@
         <v>269</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="88" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
         <v>102</v>
       </c>
@@ -4967,7 +4951,7 @@
         <v>271</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="89" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
         <v>241</v>
       </c>
@@ -4999,7 +4983,7 @@
         <v>273</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="90" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
         <v>84</v>
       </c>
@@ -5031,7 +5015,7 @@
         <v>275</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="91" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
         <v>276</v>
       </c>
@@ -5065,7 +5049,7 @@
         <v>279</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="92" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
         <v>53</v>
       </c>
@@ -5097,7 +5081,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="93" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
         <v>276</v>
       </c>
@@ -5129,7 +5113,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="94" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
         <v>92</v>
       </c>
@@ -5161,7 +5145,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="95" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
         <v>64</v>
       </c>
@@ -5195,7 +5179,7 @@
         <v>285</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="96" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
         <v>25</v>
       </c>
@@ -5227,7 +5211,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="97" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
         <v>287</v>
       </c>
@@ -5259,7 +5243,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="98" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
         <v>216</v>
       </c>
@@ -5291,7 +5275,7 @@
         <v>290</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="99" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
         <v>59</v>
       </c>
@@ -5323,7 +5307,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="100" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
         <v>276</v>
       </c>
@@ -5355,7 +5339,7 @@
         <v>39</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row r="101" spans="1:12" s="1" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
         <v>119</v>
       </c>
@@ -5393,294 +5377,184 @@
         <v>295</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75">
-      <c r="A102" s="10"/>
-      <c r="B102" s="10"/>
-      <c r="C102" s="11"/>
-      <c r="D102" s="11"/>
-      <c r="E102" s="11"/>
-      <c r="F102" s="12"/>
-      <c r="G102" s="13"/>
-      <c r="H102" s="13"/>
-      <c r="I102" s="13"/>
-      <c r="J102" s="13"/>
-      <c r="K102" s="14"/>
-      <c r="L102" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75">
-      <c r="A103" s="10"/>
-      <c r="B103" s="10"/>
-      <c r="C103" s="11"/>
-      <c r="D103" s="11"/>
-      <c r="E103" s="11"/>
-      <c r="F103" s="12"/>
-      <c r="G103" s="13"/>
-      <c r="H103" s="13"/>
-      <c r="I103" s="13"/>
-      <c r="J103" s="13"/>
-      <c r="K103" s="14"/>
-      <c r="L103" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75">
-      <c r="A104" s="15" t="s">
+    <row r="102" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="103" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="104" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A104" s="13" t="s">
         <v>296</v>
       </c>
-      <c r="B104" s="10"/>
-      <c r="C104" s="11"/>
-      <c r="D104" s="11"/>
-      <c r="E104" s="11"/>
-      <c r="F104" s="12"/>
-      <c r="G104" s="13"/>
-      <c r="H104" s="13"/>
-      <c r="I104" s="13"/>
-      <c r="J104" s="13"/>
-      <c r="K104" s="14"/>
-      <c r="L104" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75">
-      <c r="A105" s="16" t="s">
+    </row>
+    <row r="105" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A105" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B105" s="16" t="s">
+      <c r="B105" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="C105" s="16" t="s">
+      <c r="C105" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="D105" s="16" t="s">
+      <c r="D105" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="E105" s="16" t="s">
+      <c r="E105" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="F105" s="17" t="s">
+      <c r="F105" s="15" t="s">
         <v>301</v>
       </c>
-      <c r="G105" s="13"/>
-      <c r="H105" s="13"/>
-      <c r="I105" s="13"/>
-      <c r="J105" s="13"/>
-      <c r="K105" s="14"/>
-      <c r="L105" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75">
+    </row>
+    <row r="106" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="10" t="s">
         <v>302</v>
       </c>
       <c r="B106" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C106" s="18">
+      <c r="C106" s="16">
         <v>46</v>
       </c>
-      <c r="D106" s="18">
+      <c r="D106" s="16">
         <v>54</v>
       </c>
-      <c r="E106" s="18">
+      <c r="E106" s="16">
         <v>100</v>
       </c>
-      <c r="F106" s="12" t="s">
+      <c r="F106" t="s">
         <v>304</v>
       </c>
-      <c r="G106" s="13"/>
-      <c r="H106" s="13"/>
-      <c r="I106" s="13"/>
-      <c r="J106" s="13"/>
-      <c r="K106" s="14"/>
-      <c r="L106" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75">
+    </row>
+    <row r="107" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="10" t="s">
         <v>302</v>
       </c>
       <c r="B107" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C107" s="18">
+      <c r="C107" s="16">
         <v>33</v>
       </c>
-      <c r="D107" s="18">
-        <v>17</v>
-      </c>
-      <c r="E107" s="18">
+      <c r="D107" s="16">
+        <v>17</v>
+      </c>
+      <c r="E107" s="16">
         <v>50</v>
       </c>
-      <c r="F107" s="12" t="s">
+      <c r="F107" t="s">
         <v>305</v>
       </c>
-      <c r="G107" s="13"/>
-      <c r="H107" s="13"/>
-      <c r="I107" s="13"/>
-      <c r="J107" s="13"/>
-      <c r="K107" s="14"/>
-      <c r="L107" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75">
+    </row>
+    <row r="108" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="10" t="s">
         <v>302</v>
       </c>
       <c r="B108" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C108" s="18">
+      <c r="C108" s="16">
         <v>13</v>
       </c>
-      <c r="D108" s="18">
+      <c r="D108" s="16">
         <v>37</v>
       </c>
-      <c r="E108" s="18">
+      <c r="E108" s="16">
         <v>50</v>
       </c>
-      <c r="F108" s="12" t="s">
+      <c r="F108" t="s">
         <v>306</v>
       </c>
-      <c r="G108" s="13"/>
-      <c r="H108" s="13"/>
-      <c r="I108" s="13"/>
-      <c r="J108" s="13"/>
-      <c r="K108" s="14"/>
-      <c r="L108" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75">
+    </row>
+    <row r="109" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="10" t="s">
         <v>307</v>
       </c>
       <c r="B109" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C109" s="18">
+      <c r="C109" s="16">
         <v>35</v>
       </c>
-      <c r="D109" s="18">
+      <c r="D109" s="16">
         <v>65</v>
       </c>
-      <c r="E109" s="18">
+      <c r="E109" s="16">
         <v>100</v>
       </c>
-      <c r="F109" s="12" t="s">
+      <c r="F109" t="s">
         <v>308</v>
       </c>
-      <c r="G109" s="13"/>
-      <c r="H109" s="13"/>
-      <c r="I109" s="13"/>
-      <c r="J109" s="13"/>
-      <c r="K109" s="14"/>
-      <c r="L109" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75">
+    </row>
+    <row r="110" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="10" t="s">
         <v>307</v>
       </c>
       <c r="B110" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C110" s="18">
+      <c r="C110" s="16">
         <v>27</v>
       </c>
-      <c r="D110" s="18">
+      <c r="D110" s="16">
         <v>23</v>
       </c>
-      <c r="E110" s="18">
+      <c r="E110" s="16">
         <v>50</v>
       </c>
-      <c r="F110" s="12" t="s">
+      <c r="F110" t="s">
         <v>309</v>
       </c>
-      <c r="G110" s="13"/>
-      <c r="H110" s="13"/>
-      <c r="I110" s="13"/>
-      <c r="J110" s="13"/>
-      <c r="K110" s="14"/>
-      <c r="L110" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75">
+    </row>
+    <row r="111" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="10" t="s">
         <v>307</v>
       </c>
       <c r="B111" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C111" s="18">
+      <c r="C111" s="16">
         <v>8</v>
       </c>
-      <c r="D111" s="18">
+      <c r="D111" s="16">
         <v>42</v>
       </c>
-      <c r="E111" s="18">
+      <c r="E111" s="16">
         <v>50</v>
       </c>
-      <c r="F111" s="12" t="s">
+      <c r="F111" t="s">
         <v>310</v>
       </c>
-      <c r="G111" s="13"/>
-      <c r="H111" s="13"/>
-      <c r="I111" s="13"/>
-      <c r="J111" s="13"/>
-      <c r="K111" s="14"/>
-      <c r="L111" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75">
-      <c r="A112" s="10"/>
-      <c r="B112" s="10"/>
-      <c r="C112" s="11"/>
-      <c r="D112" s="11"/>
-      <c r="E112" s="11"/>
-      <c r="F112" s="12"/>
-      <c r="G112" s="13"/>
-      <c r="H112" s="13"/>
-      <c r="I112" s="13"/>
-      <c r="J112" s="13"/>
-      <c r="K112" s="14"/>
-      <c r="L112" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75">
-      <c r="A113" s="15" t="s">
+    </row>
+    <row r="112" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="113" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A113" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="B113" s="10"/>
-      <c r="C113" s="11"/>
-      <c r="D113" s="11"/>
-      <c r="E113" s="11"/>
-      <c r="F113" s="12"/>
-      <c r="G113" s="13"/>
-      <c r="H113" s="13"/>
-      <c r="I113" s="13"/>
-      <c r="J113" s="13"/>
-      <c r="K113" s="14"/>
-      <c r="L113" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75">
-      <c r="A114" s="16" t="s">
+    </row>
+    <row r="114" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B114" s="16" t="s">
+      <c r="B114" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="C114" s="16" t="s">
+      <c r="C114" s="14" t="s">
         <v>312</v>
       </c>
-      <c r="D114" s="16" t="s">
+      <c r="D114" s="14" t="s">
         <v>313</v>
       </c>
-      <c r="E114" s="16" t="s">
+      <c r="E114" s="14" t="s">
         <v>314</v>
       </c>
-      <c r="F114" s="12"/>
-      <c r="G114" s="13"/>
-      <c r="H114" s="13"/>
-      <c r="I114" s="13"/>
-      <c r="J114" s="13"/>
-      <c r="K114" s="14"/>
-      <c r="L114" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75">
+    </row>
+    <row r="115" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="10" t="s">
         <v>302</v>
       </c>
       <c r="B115" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C115" s="18">
+      <c r="C115" s="16">
         <v>87</v>
       </c>
       <c r="D115" s="11" t="s">
@@ -5689,22 +5563,15 @@
       <c r="E115" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="F115" s="12"/>
-      <c r="G115" s="13"/>
-      <c r="H115" s="13"/>
-      <c r="I115" s="13"/>
-      <c r="J115" s="13"/>
-      <c r="K115" s="14"/>
-      <c r="L115" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75">
+    </row>
+    <row r="116" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="10" t="s">
         <v>302</v>
       </c>
       <c r="B116" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C116" s="18">
+      <c r="C116" s="16">
         <v>51</v>
       </c>
       <c r="D116" s="11" t="s">
@@ -5713,22 +5580,15 @@
       <c r="E116" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="F116" s="12"/>
-      <c r="G116" s="13"/>
-      <c r="H116" s="13"/>
-      <c r="I116" s="13"/>
-      <c r="J116" s="13"/>
-      <c r="K116" s="14"/>
-      <c r="L116" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75">
+    </row>
+    <row r="117" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="10" t="s">
         <v>302</v>
       </c>
       <c r="B117" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C117" s="18">
+      <c r="C117" s="16">
         <v>36</v>
       </c>
       <c r="D117" s="11" t="s">
@@ -5737,22 +5597,15 @@
       <c r="E117" s="11" t="s">
         <v>320</v>
       </c>
-      <c r="F117" s="12"/>
-      <c r="G117" s="13"/>
-      <c r="H117" s="13"/>
-      <c r="I117" s="13"/>
-      <c r="J117" s="13"/>
-      <c r="K117" s="14"/>
-      <c r="L117" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75">
+    </row>
+    <row r="118" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="10" t="s">
         <v>307</v>
       </c>
       <c r="B118" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="C118" s="18">
+      <c r="C118" s="16">
         <v>49</v>
       </c>
       <c r="D118" s="11" t="s">
@@ -5761,22 +5614,15 @@
       <c r="E118" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="F118" s="12"/>
-      <c r="G118" s="13"/>
-      <c r="H118" s="13"/>
-      <c r="I118" s="13"/>
-      <c r="J118" s="13"/>
-      <c r="K118" s="14"/>
-      <c r="L118" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75">
+    </row>
+    <row r="119" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="10" t="s">
         <v>307</v>
       </c>
       <c r="B119" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="C119" s="18">
+      <c r="C119" s="16">
         <v>31</v>
       </c>
       <c r="D119" s="11" t="s">
@@ -5785,22 +5631,15 @@
       <c r="E119" s="11" t="s">
         <v>318</v>
       </c>
-      <c r="F119" s="12"/>
-      <c r="G119" s="13"/>
-      <c r="H119" s="13"/>
-      <c r="I119" s="13"/>
-      <c r="J119" s="13"/>
-      <c r="K119" s="14"/>
-      <c r="L119" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75">
+    </row>
+    <row r="120" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="10" t="s">
         <v>307</v>
       </c>
       <c r="B120" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="C120" s="18">
+      <c r="C120" s="16">
         <v>18</v>
       </c>
       <c r="D120" s="11" t="s">
@@ -5809,161 +5648,74 @@
       <c r="E120" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="F120" s="12"/>
-      <c r="G120" s="13"/>
-      <c r="H120" s="13"/>
-      <c r="I120" s="13"/>
-      <c r="J120" s="13"/>
-      <c r="K120" s="14"/>
-      <c r="L120" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75">
-      <c r="A121" s="10"/>
-      <c r="B121" s="10"/>
-      <c r="C121" s="11"/>
-      <c r="D121" s="11"/>
-      <c r="E121" s="11"/>
-      <c r="F121" s="12"/>
-      <c r="G121" s="13"/>
-      <c r="H121" s="13"/>
-      <c r="I121" s="13"/>
-      <c r="J121" s="13"/>
-      <c r="K121" s="14"/>
-      <c r="L121" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75">
-      <c r="A122" s="15" t="s">
+    </row>
+    <row r="121" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="122" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A122" s="13" t="s">
         <v>325</v>
       </c>
-      <c r="B122" s="10"/>
-      <c r="C122" s="11"/>
-      <c r="D122" s="11"/>
-      <c r="E122" s="11"/>
-      <c r="F122" s="12"/>
-      <c r="G122" s="13"/>
-      <c r="H122" s="13"/>
-      <c r="I122" s="13"/>
-      <c r="J122" s="13"/>
-      <c r="K122" s="14"/>
-      <c r="L122" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75">
-      <c r="A123" s="16" t="s">
+    </row>
+    <row r="123" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A123" s="14" t="s">
         <v>326</v>
       </c>
-      <c r="B123" s="16" t="s">
+      <c r="B123" s="14" t="s">
         <v>327</v>
       </c>
-      <c r="C123" s="16" t="s">
+      <c r="C123" s="14" t="s">
         <v>328</v>
       </c>
-      <c r="D123" s="16" t="s">
+      <c r="D123" s="14" t="s">
         <v>329</v>
       </c>
-      <c r="E123" s="16" t="s">
+      <c r="E123" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="F123" s="12"/>
-      <c r="G123" s="13"/>
-      <c r="H123" s="13"/>
-      <c r="I123" s="13"/>
-      <c r="J123" s="13"/>
-      <c r="K123" s="14"/>
-      <c r="L123" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75">
-      <c r="A124" s="18">
+    </row>
+    <row r="124" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A124" s="16">
         <v>34</v>
       </c>
-      <c r="B124" s="18">
+      <c r="B124" s="16">
         <v>53</v>
       </c>
-      <c r="C124" s="18">
+      <c r="C124" s="16">
         <v>13</v>
       </c>
       <c r="D124" s="11" t="s">
         <v>331</v>
       </c>
-      <c r="E124" s="18">
+      <c r="E124" s="16">
         <v>100</v>
       </c>
-      <c r="F124" s="12"/>
-      <c r="G124" s="13"/>
-      <c r="H124" s="13"/>
-      <c r="I124" s="13"/>
-      <c r="J124" s="13"/>
-      <c r="K124" s="14"/>
-      <c r="L124" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75">
-      <c r="A125" s="10"/>
-      <c r="B125" s="10"/>
-      <c r="C125" s="11"/>
-      <c r="D125" s="11"/>
-      <c r="E125" s="11"/>
-      <c r="F125" s="12"/>
-      <c r="G125" s="13"/>
-      <c r="H125" s="13"/>
-      <c r="I125" s="13"/>
-      <c r="J125" s="13"/>
-      <c r="K125" s="14"/>
-      <c r="L125" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75">
-      <c r="A126" s="15" t="s">
+    </row>
+    <row r="125" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="126" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A126" s="13" t="s">
         <v>332</v>
       </c>
-      <c r="B126" s="10"/>
-      <c r="C126" s="11"/>
-      <c r="D126" s="11"/>
-      <c r="E126" s="11"/>
-      <c r="F126" s="12"/>
-      <c r="G126" s="13"/>
-      <c r="H126" s="13"/>
-      <c r="I126" s="13"/>
-      <c r="J126" s="13"/>
-      <c r="K126" s="14"/>
-      <c r="L126" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75">
-      <c r="A127" s="16" t="s">
+    </row>
+    <row r="127" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="14" t="s">
         <v>333</v>
       </c>
-      <c r="B127" s="16" t="s">
+      <c r="B127" s="14" t="s">
         <v>334</v>
       </c>
-      <c r="C127" s="16" t="s">
+      <c r="C127" s="14" t="s">
         <v>335</v>
       </c>
-      <c r="D127" s="11"/>
-      <c r="E127" s="11"/>
-      <c r="F127" s="12"/>
-      <c r="G127" s="13"/>
-      <c r="H127" s="13"/>
-      <c r="I127" s="13"/>
-      <c r="J127" s="13"/>
-      <c r="K127" s="14"/>
-      <c r="L127" s="13"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75">
-      <c r="A128" s="18">
+    </row>
+    <row r="128" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="16">
         <v>34</v>
       </c>
-      <c r="B128" s="18">
+      <c r="B128" s="16">
         <v>31</v>
       </c>
       <c r="C128" s="11" t="s">
         <v>336</v>
       </c>
-      <c r="D128" s="11"/>
-      <c r="E128" s="11"/>
-      <c r="F128" s="12"/>
-      <c r="G128" s="13"/>
-      <c r="H128" s="13"/>
-      <c r="I128" s="13"/>
-      <c r="J128" s="13"/>
-      <c r="K128" s="14"/>
-      <c r="L128" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>